<commit_message>
turnos hospitalizados pre inteactivos
</commit_message>
<xml_diff>
--- a/Template_Ejecutivos_CEM.xlsx
+++ b/Template_Ejecutivos_CEM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECH\Desktop\Desarrollos\TurnosCLA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECH\Desktop\Desarrollos\TurnosCLA\v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{827DB70E-5186-4D27-A0B4-E82E24DCC0C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7FFAF6-5E45-4B48-AF29-989E75AF3A60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-11100" windowWidth="16440" windowHeight="28320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demanda" sheetId="3" r:id="rId1"/>
@@ -2093,7 +2093,7 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C6" t="s">
         <v>9</v>
@@ -2104,7 +2104,7 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
         <v>9</v>

</xml_diff>